<commit_message>
_ correct import with type
</commit_message>
<xml_diff>
--- a/laravel_app/database/import_post.xlsx
+++ b/laravel_app/database/import_post.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A94B3E15-297D-7D45-A6F5-ABA969D90B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334E2A09-337D-BE47-8C62-36E81AA438EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-45820" yWindow="-380" windowWidth="25260" windowHeight="17500" xr2:uid="{CBB3C014-C24F-6540-AB8C-3313D5389319}"/>
+    <workbookView xWindow="-29520" yWindow="-440" windowWidth="25260" windowHeight="17500" xr2:uid="{CBB3C014-C24F-6540-AB8C-3313D5389319}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="87">
   <si>
     <t>STT</t>
   </si>
@@ -106,9 +106,6 @@
     <t>Hợp Đồng lao động</t>
   </si>
   <si>
-    <t>Hợp đông lao động</t>
-  </si>
-  <si>
     <t>Thời gian làm việc</t>
   </si>
   <si>
@@ -227,6 +224,78 @@
   </si>
   <si>
     <t>POS241105000002</t>
+  </si>
+  <si>
+    <t>Mua móng</t>
+  </si>
+  <si>
+    <t>tại gia</t>
+  </si>
+  <si>
+    <t>POS241105000003</t>
+  </si>
+  <si>
+    <t>POS241105000004</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>Recruitment</t>
+  </si>
+  <si>
+    <t>Find Job</t>
+  </si>
+  <si>
+    <t>Nail</t>
+  </si>
+  <si>
+    <t>Cần tuyền thợ naill</t>
+  </si>
+  <si>
+    <t>Cần tìm việc nail</t>
+  </si>
+  <si>
+    <t>Đang cần tuyển thợ nail ở tiểu bang cali</t>
+  </si>
+  <si>
+    <t>Cần tìm việc ở bang Cali</t>
+  </si>
+  <si>
+    <t>0909111112</t>
+  </si>
+  <si>
+    <t>0909112234</t>
+  </si>
+  <si>
+    <t>viec_nail@nail.com</t>
+  </si>
+  <si>
+    <t>tim_viec@nail.com</t>
+  </si>
+  <si>
+    <t>Cali 2 nail</t>
+  </si>
+  <si>
+    <t>99 Hồ Tùng Mậu</t>
+  </si>
+  <si>
+    <t>Làm tại bàn</t>
+  </si>
+  <si>
+    <t>full time</t>
+  </si>
+  <si>
+    <t>2 năm</t>
+  </si>
+  <si>
+    <t>T2, T3, T4, T5</t>
+  </si>
+  <si>
+    <t>1 năm</t>
+  </si>
+  <si>
+    <t>part time</t>
   </si>
 </sst>
 </file>
@@ -590,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85A7B3D-51C4-A149-BF30-6E5B51BE25F5}">
-  <dimension ref="A1:AN3"/>
+  <dimension ref="A1:AM5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -599,7 +668,7 @@
     <col min="15" max="15" width="11.1640625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -717,108 +786,232 @@
       <c r="AM1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s">
-        <v>39</v>
-      </c>
     </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
         <v>40</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
         <v>41</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>42</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>43</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" t="s">
         <v>46</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
+        <v>48</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="P2" t="s">
         <v>47</v>
       </c>
-      <c r="M2" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="P2" t="s">
-        <v>48</v>
-      </c>
-      <c r="AK2">
+      <c r="AC2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AJ2">
         <v>2000000</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" t="s">
         <v>63</v>
       </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E3">
+      <c r="M3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="P3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AJ3">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:39" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4">
         <v>1</v>
       </c>
-      <c r="F3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L4" t="s">
+        <v>79</v>
+      </c>
+      <c r="M4" t="s">
+        <v>80</v>
+      </c>
+      <c r="N4" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="P3" t="s">
-        <v>57</v>
-      </c>
-      <c r="AK3">
-        <v>1500000</v>
+      <c r="P4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>81</v>
+      </c>
+      <c r="R4">
+        <v>800</v>
+      </c>
+      <c r="S4">
+        <v>800</v>
+      </c>
+      <c r="T4">
+        <v>2500</v>
+      </c>
+      <c r="U4">
+        <v>1</v>
+      </c>
+      <c r="V4" t="s">
+        <v>82</v>
+      </c>
+      <c r="W4" t="s">
+        <v>83</v>
+      </c>
+      <c r="X4" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:39" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" t="s">
+        <v>74</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="R5">
+        <v>1200</v>
+      </c>
+      <c r="U5">
+        <v>2</v>
+      </c>
+      <c r="V5" t="s">
+        <v>86</v>
+      </c>
+      <c r="W5" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y5">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -826,6 +1019,8 @@
     <hyperlink ref="J2" r:id="rId1" xr:uid="{21026F74-9542-CF42-966B-1685C2322541}"/>
     <hyperlink ref="K2" r:id="rId2" xr:uid="{8747D9CB-B5EF-E041-82D7-85D8C2B48E78}"/>
     <hyperlink ref="J3" r:id="rId3" xr:uid="{49BFE669-E797-504E-9D17-1E687B43FB33}"/>
+    <hyperlink ref="J4" r:id="rId4" xr:uid="{A431C32E-7B1B-2746-9D0E-1E0462B9A16B}"/>
+    <hyperlink ref="J5" r:id="rId5" xr:uid="{CD2DD1FD-C459-2D48-B91D-A05EEFE094B8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>